<commit_message>
chore: sync Excel watchlist with CAN_SLIM_CLAUDE.md (1 Jun 2026)
Add VISN #1, YOU #2, AGX #3, COCO #4 as new watchlist rows.
Update AUPH and PAYS to conditional watchlist (trigger: RS≥85).
Remove old #1-#4 numbering from ABX, DDI, OPRA, VOXR.
Update header subtitle with new active watchlist.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAN_SLIM_Tracker_updated.xlsx
+++ b/CAN_SLIM_Tracker_updated.xlsx
@@ -1261,7 +1261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE24"/>
+  <dimension ref="A1:AE28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="72" min="1" max="1"/>
@@ -1291,7 +1291,7 @@
     <row r="2" ht="39.75" customHeight="1" s="72">
       <c r="A2" s="73" t="inlineStr">
         <is>
-          <t>Última revisión completa: 30 Mayo 2026 | Watchlist activa: PAYS #1 · ABX #2 · DDI #3 · OPRA #4 · VOXR</t>
+          <t>Última revisión: 2026-06-01 | Watchlist activa: VISN #1 · YOU #2 · AGX #3 · COCO #4 · AUPH (cond.) · PAYS (cond.)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="Y8" s="157" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST #1</t>
+          <t>👀 WATCHLIST</t>
         </is>
       </c>
       <c r="Z8" s="101">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="AE8" s="158" t="inlineStr">
         <is>
-          <t>[30may26] MEJOR CANDIDATO. Revenue +50.8% YoY real sin one-times. D/E 0.11. ROE 22%, Margin 11%. Pivot $8.88. RS 67 único freno. Vol 960K borderline.</t>
+          <t>[1jun26] RS 71 — condicional. Activar cuando RS ≥ 85 Y vol promedio &gt; 1M. Trigger breakout $8.88 con vol.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="Y9" s="159" t="inlineStr">
         <is>
-          <t>🚫 DESCARTAR</t>
+          <t>👀 WATCHLIST</t>
         </is>
       </c>
       <c r="Z9" s="129">
@@ -1891,12 +1891,12 @@
       </c>
       <c r="AD9" s="132" t="inlineStr">
         <is>
-          <t>Reevaluar en 2T si rev &gt;25%</t>
+          <t>Semanal. Monitorear RS</t>
         </is>
       </c>
       <c r="AE9" s="160" t="inlineStr">
         <is>
-          <t>[30may26] Revenue +24% borderline. Guidance FY26 +11-15% (desaceleración). CEO+COO+CFO reemplazados en mar26. R/R 0.6x. Upside analistas solo +12.9%.</t>
+          <t>[1jun26] RS 82 — condicional. Activar cuando RS ≥ 85 → analizar con Claude.</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="Y18" s="171" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST #2</t>
+          <t>👀 WATCHLIST</t>
         </is>
       </c>
       <c r="Z18" s="103">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="Y20" s="171" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST #3</t>
+          <t>👀 WATCHLIST</t>
         </is>
       </c>
       <c r="Z20" s="103">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="Y22" s="171" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST #4</t>
+          <t>👀 WATCHLIST</t>
         </is>
       </c>
       <c r="Z22" s="103">
@@ -3420,47 +3420,315 @@
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="72">
-      <c r="A23" s="95" t="n"/>
-      <c r="B23" s="94" t="n"/>
-      <c r="C23" s="95" t="n"/>
-      <c r="D23" s="95" t="n"/>
-      <c r="E23" s="95" t="n"/>
-      <c r="F23" s="84" t="n"/>
-      <c r="G23" s="84" t="n"/>
-      <c r="H23" s="84" t="n"/>
-      <c r="I23" s="103" t="n"/>
-      <c r="J23" s="96" t="n"/>
-      <c r="K23" s="95" t="n"/>
-      <c r="L23" s="96" t="n"/>
-      <c r="M23" s="96" t="n"/>
-      <c r="N23" s="96" t="n"/>
-      <c r="O23" s="97" t="n"/>
-      <c r="P23" s="95" t="n"/>
-      <c r="Q23" s="96" t="n"/>
-      <c r="R23" s="96" t="n"/>
-      <c r="S23" s="95" t="n"/>
-      <c r="T23" s="103" t="n"/>
-      <c r="U23" s="103" t="n"/>
-      <c r="V23" s="103" t="n"/>
-      <c r="W23" s="103" t="n"/>
-      <c r="X23" s="103" t="n"/>
-      <c r="Y23" s="103" t="n"/>
-      <c r="Z23" s="103" t="n"/>
-      <c r="AA23" s="103" t="n"/>
-      <c r="AC23" s="103" t="n"/>
-      <c r="AE23" s="95" t="n"/>
+      <c r="A23" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="P23" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="T23" s="0" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="U23" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V23" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W23" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X23" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y23" s="0" t="inlineStr">
+        <is>
+          <t>👀 WATCHLIST #1</t>
+        </is>
+      </c>
+      <c r="AD23" s="0" t="inlineStr">
+        <is>
+          <t>Alerta $12.80 vol≥10.6M</t>
+        </is>
+      </c>
+      <c r="AE23" s="0" t="inlineStr">
+        <is>
+          <t>[1jun26] RS 99. Pendiente screener.py. Trigger: ruptura $12.80 con vol ≥ 10.6M.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="22" customHeight="1" s="72">
-      <c r="A24" s="114" t="inlineStr">
+      <c r="A24" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>99</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>👀 WATCHLIST #2</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Alerta breakout $62.36</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>[1jun26] RS 99. Pendiente screener.py. Trigger: breakout $62.36 con vol ≥ 50% promedio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="72">
+      <c r="A25" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>AGX</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="P25" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="T25" s="0" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="U25" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V25" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W25" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X25" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y25" s="0" t="inlineStr">
+        <is>
+          <t>👀 WATCHLIST #3</t>
+        </is>
+      </c>
+      <c r="AD25" s="0" t="inlineStr">
+        <is>
+          <t>Alerta breakout $740.91</t>
+        </is>
+      </c>
+      <c r="AE25" s="0" t="inlineStr">
+        <is>
+          <t>[1jun26] RS 99. Pendiente screener.py. Trigger: breakout $740.91 con vol ≥ 500K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="72">
+      <c r="A26" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>COCO</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="P26" s="0" t="n">
+        <v>93</v>
+      </c>
+      <c r="T26" s="0" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="U26" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V26" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W26" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X26" s="0" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y26" s="0" t="inlineStr">
+        <is>
+          <t>👀 WATCHLIST #4</t>
+        </is>
+      </c>
+      <c r="AD26" s="0" t="inlineStr">
+        <is>
+          <t>Pullback SMA50 ~$60.68</t>
+        </is>
+      </c>
+      <c r="AE26" s="0" t="inlineStr">
+        <is>
+          <t>[1jun26] RS 93. Pendiente screener.py. Esperar pullback a SMA50 ~$60.68.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="72">
+      <c r="A27" s="95" t="n"/>
+      <c r="B27" s="94" t="n"/>
+      <c r="C27" s="95" t="n"/>
+      <c r="D27" s="95" t="n"/>
+      <c r="E27" s="95" t="n"/>
+      <c r="F27" s="84" t="n"/>
+      <c r="G27" s="84" t="n"/>
+      <c r="H27" s="84" t="n"/>
+      <c r="I27" s="103" t="n"/>
+      <c r="J27" s="96" t="n"/>
+      <c r="K27" s="95" t="n"/>
+      <c r="L27" s="96" t="n"/>
+      <c r="M27" s="96" t="n"/>
+      <c r="N27" s="96" t="n"/>
+      <c r="O27" s="97" t="n"/>
+      <c r="P27" s="95" t="n"/>
+      <c r="Q27" s="96" t="n"/>
+      <c r="R27" s="96" t="n"/>
+      <c r="S27" s="95" t="n"/>
+      <c r="T27" s="103" t="n"/>
+      <c r="U27" s="103" t="n"/>
+      <c r="V27" s="103" t="n"/>
+      <c r="W27" s="103" t="n"/>
+      <c r="X27" s="103" t="n"/>
+      <c r="Y27" s="103" t="n"/>
+      <c r="Z27" s="103" t="n"/>
+      <c r="AA27" s="103" t="n"/>
+      <c r="AC27" s="103" t="n"/>
+      <c r="AE27" s="95" t="n"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="72">
+      <c r="A28" s="114" t="inlineStr">
         <is>
           <t>📌 LEYENDA  |  🔵 Azul = INPUTS manuales  |  ⚫ Negro = Fórmulas  |  🟢 OPERAR ≥3.5/4  |  🟡 WATCHLIST 2.5–3/4  |  🔴 NO OPERAR &lt;2.5  |  🚫 DESCARTAR: Falla F1</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="72"/>
-    <row r="26" ht="15.75" customHeight="1" s="72"/>
-    <row r="27" ht="15.75" customHeight="1" s="72"/>
-    <row r="28" ht="15.75" customHeight="1" s="72"/>
     <row r="29" ht="15.75" customHeight="1" s="72"/>
     <row r="30" ht="15.75" customHeight="1" s="72"/>
     <row r="31" ht="15.75" customHeight="1" s="72"/>
@@ -4434,12 +4702,11 @@
     <row r="999" ht="15.75" customHeight="1" s="72"/>
     <row r="1000" ht="15.75" customHeight="1" s="72"/>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="A4:AE4"/>
     <mergeCell ref="T5:Y5"/>
     <mergeCell ref="J5:O5"/>
     <mergeCell ref="A2:AE2"/>
-    <mergeCell ref="A24:AE24"/>
     <mergeCell ref="P5:R5"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="AD5:AE5"/>

</xml_diff>

<commit_message>
chore: fill Excel columns for YOU, AGX, COCO from 2026-06-01 reports
YOU: Clear Secure — EPS +52.7%, ROE 109.5%, RS 99, F2 4/4, F3 2/3
AGX: Argan — EPS +56.9%, ROE 33.8%, RS 99, F2 4/4, F3 2/3, vol insuficiente
COCO: Vita Coco — EPS +61.4%, ROE 26.3%, RS 93, F2 3/4, F3 2/3, sobreextendida
VISN: sin reporte disponible, pendiente screener.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAN_SLIM_Tracker_updated.xlsx
+++ b/CAN_SLIM_Tracker_updated.xlsx
@@ -3483,7 +3483,7 @@
       </c>
       <c r="AE23" s="0" t="inlineStr">
         <is>
-          <t>[1jun26] RS 99. Pendiente screener.py. Trigger: ruptura $12.80 con vol ≥ 10.6M.</t>
+          <t>[1jun26] RS 99. Sin reporte screener.py disponible. Trigger: ruptura $12.80 con vol ≥ 10.6M. Pendiente análisis fundamental completo.</t>
         </is>
       </c>
     </row>
@@ -3491,67 +3491,97 @@
       <c r="A24" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>YOU</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Clear Secure, Inc.</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="H24" t="n">
+        <v>40.34</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.095</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="P24" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="S24" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="T24" s="0" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="U24" s="0" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="V24" s="0" t="inlineStr">
+        <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="W24" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="X24" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>99</v>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr">
+      <c r="Y24" s="0" t="inlineStr">
         <is>
           <t>👀 WATCHLIST #2</t>
         </is>
       </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>Alerta breakout $62.36</t>
-        </is>
-      </c>
-      <c r="AE24" t="inlineStr">
-        <is>
-          <t>[1jun26] RS 99. Pendiente screener.py. Trigger: breakout $62.36 con vol ≥ 50% promedio.</t>
+      <c r="AD24" s="0" t="inlineStr">
+        <is>
+          <t>Diario. Alerta breakout $62.36 vol≥50%</t>
+        </is>
+      </c>
+      <c r="AE24" s="0" t="inlineStr">
+        <is>
+          <t>[1jun26] RS 99. EPS +52.7% YoY, ROE 109.5%, FCF 4.5%, D/E 0.52. Precio $57.1 (-8.4% de máx $62.36). Vol -65% vs prom — sin breakout. Etapa 2. Esperar vol ≥50% sobre prom 50d en quiebre de $62.36.</t>
         </is>
       </c>
     </row>
@@ -3566,22 +3596,52 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Argan, Inc.</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
+      </c>
+      <c r="F25" t="n">
+        <v>655.45</v>
+      </c>
+      <c r="G25" t="n">
+        <v>621.51</v>
+      </c>
+      <c r="H25" t="n">
+        <v>400.54</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.01</v>
       </c>
       <c r="P25" s="0" t="n">
         <v>99</v>
       </c>
+      <c r="Q25" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="R25" t="n">
+        <v>-0.278</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0.421</v>
+      </c>
       <c r="T25" s="0" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3589,24 +3649,24 @@
       </c>
       <c r="U25" s="0" t="inlineStr">
         <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="V25" s="0" t="inlineStr">
+        <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="W25" s="0" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="V25" s="0" t="inlineStr">
+      <c r="X25" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="W25" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X25" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="Y25" s="0" t="inlineStr">
         <is>
           <t>👀 WATCHLIST #3</t>
@@ -3614,12 +3674,12 @@
       </c>
       <c r="AD25" s="0" t="inlineStr">
         <is>
-          <t>Alerta breakout $740.91</t>
+          <t>Semanal. Alerta vol &gt;500K + breakout $740.91</t>
         </is>
       </c>
       <c r="AE25" s="0" t="inlineStr">
         <is>
-          <t>[1jun26] RS 99. Pendiente screener.py. Trigger: breakout $740.91 con vol ≥ 500K.</t>
+          <t>[1jun26] RS 99. EPS +56.9% YoY, ROE 33.8%, FCF 3.7%, D/E 0.01. Vol 421K INSUFICIENTE (&lt;1M). Precio $655 (-11.5% de máx $740.91). Target analistas -27.8% (Wall St escéptico). Etapa 2. Trigger: vol &gt;500K + breakout $740.91.</t>
         </is>
       </c>
     </row>
@@ -3634,22 +3694,52 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>The Vita Coco Company, Inc.</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
+      </c>
+      <c r="F26" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="G26" t="n">
+        <v>60.68</v>
+      </c>
+      <c r="H26" t="n">
+        <v>51.01</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.04</v>
       </c>
       <c r="P26" s="0" t="n">
         <v>93</v>
       </c>
+      <c r="Q26" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="R26" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1.4</v>
+      </c>
       <c r="T26" s="0" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3657,24 +3747,24 @@
       </c>
       <c r="U26" s="0" t="inlineStr">
         <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="V26" s="0" t="inlineStr">
+        <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="W26" s="0" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="V26" s="0" t="inlineStr">
+      <c r="X26" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="W26" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X26" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="Y26" s="0" t="inlineStr">
         <is>
           <t>👀 WATCHLIST #4</t>
@@ -3682,12 +3772,12 @@
       </c>
       <c r="AD26" s="0" t="inlineStr">
         <is>
-          <t>Pullback SMA50 ~$60.68</t>
+          <t>Pullback SMA50 ~$60.68. Monitorear vol</t>
         </is>
       </c>
       <c r="AE26" s="0" t="inlineStr">
         <is>
-          <t>[1jun26] RS 93. Pendiente screener.py. Esperar pullback a SMA50 ~$60.68.</t>
+          <t>[1jun26] RS 93. EPS +61.4% YoY, ROE 26.3%, FCF 1.1% (débil), D/E 0.04. Precio $76.2 (+25.6% sobre SMA50 — sobreextendido). Vol -78.3% vs prom. Target analistas -1.4% (sin convicción). Etapa 2 tardía. Esperar pullback a SMA50 $60.68.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: fill Excel VISN from 2026-06-01 report
Vistance Networks — EPS +602.6%, RS 99, F2 3/4, F3 3/3
Sales 21.6% débil, ROE 13.1% débil, FCF 27%
Trigger: ruptura $12.80 con vol ≥ 10.6M

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAN_SLIM_Tracker_updated.xlsx
+++ b/CAN_SLIM_Tracker_updated.xlsx
@@ -3430,47 +3430,77 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Vistance Networks, Inc.</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
+      </c>
+      <c r="F23" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="G23" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="H23" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="M23" t="n">
+        <v>3.477</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.01</v>
       </c>
       <c r="P23" s="0" t="n">
         <v>99</v>
       </c>
+      <c r="Q23" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="S23" t="n">
+        <v>6.7</v>
+      </c>
       <c r="T23" s="0" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="U23" s="0" t="inlineStr">
         <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="V23" s="0" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="W23" s="0" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="V23" s="0" t="inlineStr">
+      <c r="X23" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="W23" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X23" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="Y23" s="0" t="inlineStr">
         <is>
           <t>👀 WATCHLIST #1</t>
@@ -3478,12 +3508,12 @@
       </c>
       <c r="AD23" s="0" t="inlineStr">
         <is>
-          <t>Alerta $12.80 vol≥10.6M</t>
+          <t>Diario. Alerta ruptura $12.80 vol≥10.6M</t>
         </is>
       </c>
       <c r="AE23" s="0" t="inlineStr">
         <is>
-          <t>[1jun26] RS 99. Sin reporte screener.py disponible. Trigger: ruptura $12.80 con vol ≥ 10.6M. Pendiente análisis fundamental completo.</t>
+          <t>[1jun26] RS 99. EPS +602.6% YoY, Sales +21.6% (❌&lt;25%), ROE 13.1% (❌&lt;17%), FCF 27%, D/E 0.01. F3 3/3 (único). Precio $12.39 (-3.2% de máx $12.80). Vol -59.1% — sin breakout. Etapa 2 tardía, riesgo Etapa 3. Trigger: ruptura $12.80 con vol ≥ 10.6M.</t>
         </is>
       </c>
     </row>
@@ -3511,37 +3541,37 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="0" t="n">
         <v>57.1</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" s="0" t="n">
         <v>54.6</v>
       </c>
-      <c r="H24" t="n">
+      <c r="H24" s="0" t="n">
         <v>40.34</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L24" s="0" t="n">
         <v>1.095</v>
       </c>
-      <c r="M24" t="n">
+      <c r="M24" s="0" t="n">
         <v>0.13</v>
       </c>
-      <c r="N24" t="n">
+      <c r="N24" s="0" t="n">
         <v>0.045</v>
       </c>
-      <c r="O24" t="n">
+      <c r="O24" s="0" t="n">
         <v>0.52</v>
       </c>
       <c r="P24" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="Q24" s="0" t="n">
         <v>0.97</v>
       </c>
-      <c r="R24" t="n">
+      <c r="R24" s="0" t="n">
         <v>0.08599999999999999</v>
       </c>
-      <c r="S24" t="n">
+      <c r="S24" s="0" t="n">
         <v>1.7</v>
       </c>
       <c r="T24" s="0" t="inlineStr">
@@ -3609,37 +3639,37 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="0" t="n">
         <v>655.45</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="0" t="n">
         <v>621.51</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" s="0" t="n">
         <v>400.54</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L25" s="0" t="n">
         <v>0.338</v>
       </c>
-      <c r="M25" t="n">
+      <c r="M25" s="0" t="n">
         <v>0.146</v>
       </c>
-      <c r="N25" t="n">
+      <c r="N25" s="0" t="n">
         <v>0.037</v>
       </c>
-      <c r="O25" t="n">
+      <c r="O25" s="0" t="n">
         <v>0.01</v>
       </c>
       <c r="P25" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="Q25" s="0" t="n">
         <v>1.018</v>
       </c>
-      <c r="R25" t="n">
+      <c r="R25" s="0" t="n">
         <v>-0.278</v>
       </c>
-      <c r="S25" t="n">
+      <c r="S25" s="0" t="n">
         <v>0.421</v>
       </c>
       <c r="T25" s="0" t="inlineStr">
@@ -3707,37 +3737,37 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" s="0" t="n">
         <v>76.2</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" s="0" t="n">
         <v>60.68</v>
       </c>
-      <c r="H26" t="n">
+      <c r="H26" s="0" t="n">
         <v>51.01</v>
       </c>
-      <c r="L26" t="n">
+      <c r="L26" s="0" t="n">
         <v>0.263</v>
       </c>
-      <c r="M26" t="n">
+      <c r="M26" s="0" t="n">
         <v>0.126</v>
       </c>
-      <c r="N26" t="n">
+      <c r="N26" s="0" t="n">
         <v>0.011</v>
       </c>
-      <c r="O26" t="n">
+      <c r="O26" s="0" t="n">
         <v>0.04</v>
       </c>
       <c r="P26" s="0" t="n">
         <v>93</v>
       </c>
-      <c r="Q26" t="n">
+      <c r="Q26" s="0" t="n">
         <v>0.958</v>
       </c>
-      <c r="R26" t="n">
+      <c r="R26" s="0" t="n">
         <v>-0.014</v>
       </c>
-      <c r="S26" t="n">
+      <c r="S26" s="0" t="n">
         <v>1.4</v>
       </c>
       <c r="T26" s="0" t="inlineStr">

</xml_diff>

<commit_message>
chore: rebuild Excel watchlist — 6 tickers limpios en orden de prioridad
Elimina los 16 tickers anteriores (ZVRA, VOXR, LPG, FLXS, NVGS, SPIR,
TRS, CTS, ABUS, ABX, GTY, DDI, PLGO, OPRA + duplicados).
Deja solo watchlist activa con datos completos de reportes 2026-06-01:

1. VISN — RS 99, trigger $12.80 vol≥10.6M, F2 3/4, F3 3/3
2. YOU  — RS 99, trigger $62.36 vol≥50%, F2 4/4, F3 2/3
3. AGX  — RS 99, trigger $740.91 vol≥500K, F2 4/4, F3 2/3
4. COCO — RS 93, pullback SMA50 $60.68, F2 3/4, F3 2/3
5. AUPH — RS 81, condicional RS≥85, F2 4/4, F3 1/3
6. PAYS — RS 71, condicional RS≥85 + vol>1M, F2 4/4, F3 2/3

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAN_SLIM_Tracker_updated.xlsx
+++ b/CAN_SLIM_Tracker_updated.xlsx
@@ -1261,7 +1261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE28"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="72" min="1" max="1"/>
@@ -1555,114 +1555,104 @@
       </c>
       <c r="B7" s="94" t="inlineStr">
         <is>
-          <t>ZVRA</t>
+          <t>VISN</t>
         </is>
       </c>
       <c r="C7" s="95" t="inlineStr">
         <is>
-          <t>Zevra Therapeutics</t>
+          <t>Vistance Networks, Inc.</t>
         </is>
       </c>
       <c r="D7" s="95" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E7" s="95" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F7" s="133" t="n">
-        <v>11.59</v>
+        <v>12.39</v>
       </c>
       <c r="G7" s="133" t="n">
-        <v>10.15</v>
+        <v>10.42</v>
       </c>
       <c r="H7" s="133" t="n">
-        <v>9.390000000000001</v>
-      </c>
-      <c r="I7" s="95">
-        <f>IF(G7&gt;H7,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
+        <v>8.949999999999999</v>
+      </c>
+      <c r="I7" s="95" t="n"/>
       <c r="J7" s="96" t="n">
-        <v>13.23</v>
+        <v>6.026</v>
       </c>
       <c r="K7" s="95" t="n"/>
       <c r="L7" s="96" t="n">
-        <v>0.947</v>
+        <v>0.131</v>
       </c>
       <c r="M7" s="96" t="n">
-        <v>0.84</v>
+        <v>3.477</v>
       </c>
       <c r="N7" s="96" t="n">
-        <v>0.038</v>
+        <v>0.27</v>
       </c>
       <c r="O7" s="97" t="n">
         <v>0.01</v>
       </c>
       <c r="P7" s="98" t="n">
-        <v>52</v>
+        <v>99</v>
       </c>
       <c r="Q7" s="96" t="n">
-        <v>0.707</v>
+        <v>0.976</v>
       </c>
       <c r="R7" s="96" t="n">
-        <v>0.984</v>
+        <v>0.372</v>
       </c>
       <c r="S7" s="99" t="n">
-        <v>1.4</v>
+        <v>6.7</v>
       </c>
       <c r="T7" s="134" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="U7" s="95" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="V7" s="95" t="inlineStr">
         <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="W7" s="95">
-        <f>IF(S7&gt;1,"✅ PASA",IF(S7&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X7" s="100">
-        <f>COUNTIF(T7:W7,"✅ PASA")+COUNTIF(T7:W7,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="W7" s="95" t="n"/>
+      <c r="X7" s="100" t="n"/>
       <c r="Y7" s="157" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z7" s="101">
-        <f>F7*0.93</f>
-        <v/>
-      </c>
-      <c r="AA7" s="101">
-        <f>F7*1.20</f>
-        <v/>
-      </c>
-      <c r="AB7" s="135" t="n"/>
-      <c r="AC7" s="102">
-        <f>IF(F7-Z7&lt;&gt;0,(AA7-F7)/MAX(F7-Z7,1),"-")</f>
-        <v/>
+          <t>👀 WATCHLIST #1</t>
+        </is>
+      </c>
+      <c r="Z7" s="101" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="AA7" s="101" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="AB7" s="135" t="n">
+        <v>17</v>
+      </c>
+      <c r="AC7" s="102" t="n">
+        <v>2.9</v>
       </c>
       <c r="AD7" s="136" t="inlineStr">
         <is>
-          <t>Q2 ago26. Alerta $13.00</t>
+          <t>Diario. Alerta ruptura $12.80 vol≥10.6M</t>
         </is>
       </c>
       <c r="AE7" s="158" t="inlineStr">
         <is>
-          <t>[30may26] BIOTECH EXCLUIDO. RS 52. Pivot $13.16 con vol ≥40%. Net income Q1 inflado por venta SDX ($43M one-time). Esperar RS&gt;70 + breakout real.</t>
+          <t>[1jun26] RS 99. EPS +602.6%, Sales +21.6% (❌&lt;25%), ROE 13.1% (❌&lt;17%), FCF 27%. F3 3/3 (único de la watchlist). Precio $12.39 (-3.2% de máx $12.80). Vol -59.1% — sin breakout. Etapa 2 tardía. Trigger: ruptura $12.80 con vol ≥ 10.6M.</t>
         </is>
       </c>
     </row>
@@ -1672,12 +1662,12 @@
       </c>
       <c r="B8" s="94" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>YOU</t>
         </is>
       </c>
       <c r="C8" s="95" t="inlineStr">
         <is>
-          <t>Paysign Inc</t>
+          <t>Clear Secure, Inc.</t>
         </is>
       </c>
       <c r="D8" s="95" t="inlineStr">
@@ -1687,49 +1677,46 @@
       </c>
       <c r="E8" s="95" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F8" s="133" t="n">
-        <v>7.31</v>
+        <v>57.1</v>
       </c>
       <c r="G8" s="133" t="n">
-        <v>5.97</v>
+        <v>54.6</v>
       </c>
       <c r="H8" s="133" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="I8" s="95">
-        <f>IF(G8&gt;H8,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
+        <v>40.34</v>
+      </c>
+      <c r="I8" s="95" t="n"/>
       <c r="J8" s="96" t="n">
-        <v>1.103</v>
+        <v>0.527</v>
       </c>
       <c r="K8" s="95" t="n"/>
       <c r="L8" s="96" t="n">
-        <v>0.221</v>
+        <v>1.095</v>
       </c>
       <c r="M8" s="96" t="n">
-        <v>0.114</v>
+        <v>0.13</v>
       </c>
       <c r="N8" s="96" t="n">
-        <v>0.022</v>
+        <v>0.045</v>
       </c>
       <c r="O8" s="97" t="n">
-        <v>0.11</v>
+        <v>0.52</v>
       </c>
       <c r="P8" s="98" t="n">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="Q8" s="96" t="n">
-        <v>0.473</v>
+        <v>0.97</v>
       </c>
       <c r="R8" s="96" t="n">
-        <v>0.361</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="S8" s="99" t="n">
-        <v>0.96</v>
+        <v>1.7</v>
       </c>
       <c r="T8" s="134" t="inlineStr">
         <is>
@@ -1746,40 +1733,33 @@
           <t>2/3</t>
         </is>
       </c>
-      <c r="W8" s="95">
-        <f>IF(S8&gt;1,"✅ PASA",IF(S8&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X8" s="100">
-        <f>COUNTIF(T8:W8,"✅ PASA")+COUNTIF(T8:W8,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
+      <c r="W8" s="95" t="n"/>
+      <c r="X8" s="100" t="n"/>
       <c r="Y8" s="157" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z8" s="101">
-        <f>F8*0.93</f>
-        <v/>
-      </c>
-      <c r="AA8" s="101">
-        <f>F8*1.20</f>
-        <v/>
-      </c>
-      <c r="AB8" s="135" t="n"/>
-      <c r="AC8" s="102">
-        <f>IF(F8-Z8&lt;&gt;0,(AA8-F8)/MAX(F8-Z8,1),"-")</f>
-        <v/>
+          <t>👀 WATCHLIST #2</t>
+        </is>
+      </c>
+      <c r="Z8" s="101" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="AA8" s="101" t="n">
+        <v>68.52</v>
+      </c>
+      <c r="AB8" s="135" t="n">
+        <v>62</v>
+      </c>
+      <c r="AC8" s="102" t="n">
+        <v>2.9</v>
       </c>
       <c r="AD8" s="136" t="inlineStr">
         <is>
-          <t>Semanal. Alerta $8.50–$8.88</t>
+          <t>Diario. Alerta breakout $62.36 vol≥50%</t>
         </is>
       </c>
       <c r="AE8" s="158" t="inlineStr">
         <is>
-          <t>[1jun26] RS 71 — condicional. Activar cuando RS ≥ 85 Y vol promedio &gt; 1M. Trigger breakout $8.88 con vol.</t>
+          <t>[1jun26] RS 99. EPS +52.7%, ROE 109.5%, FCF 4.5%, D/E 0.52. F2 4/4. Precio $57.1 (-8.4% de máx $62.36). Vol -65% vs prom — sin breakout. Etapa 2. Esperar vol ≥50% sobre prom 50d en quiebre de $62.36.</t>
         </is>
       </c>
     </row>
@@ -1789,68 +1769,65 @@
       </c>
       <c r="B9" s="121" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>AGX</t>
         </is>
       </c>
       <c r="C9" s="120" t="inlineStr">
         <is>
-          <t>Aurinia Pharmaceuticals</t>
+          <t>Argan, Inc.</t>
         </is>
       </c>
       <c r="D9" s="120" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="E9" s="120" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F9" s="122" t="n">
-        <v>15.06</v>
+        <v>655.45</v>
       </c>
       <c r="G9" s="122" t="n">
-        <v>15.49</v>
+        <v>621.51</v>
       </c>
       <c r="H9" s="122" t="n">
-        <v>14.32</v>
-      </c>
-      <c r="I9" s="120">
-        <f>IF(G9&gt;H9,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
+        <v>400.54</v>
+      </c>
+      <c r="I9" s="120" t="n"/>
       <c r="J9" s="123" t="n">
-        <v>0.472</v>
+        <v>0.569</v>
       </c>
       <c r="K9" s="120" t="n"/>
       <c r="L9" s="123" t="n">
-        <v>0.65</v>
+        <v>0.338</v>
       </c>
       <c r="M9" s="123" t="n">
-        <v>1</v>
+        <v>0.146</v>
       </c>
       <c r="N9" s="123" t="n">
-        <v>0.064</v>
+        <v>0.037</v>
       </c>
       <c r="O9" s="124" t="n">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="P9" s="125" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="Q9" s="123" t="n">
-        <v>0.594</v>
+        <v>1.018</v>
       </c>
       <c r="R9" s="123" t="n">
-        <v>0.129</v>
+        <v>-0.278</v>
       </c>
       <c r="S9" s="126" t="n">
-        <v>1.2</v>
+        <v>0.421</v>
       </c>
       <c r="T9" s="127" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="U9" s="120" t="inlineStr">
@@ -1860,43 +1837,36 @@
       </c>
       <c r="V9" s="120" t="inlineStr">
         <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W9" s="120">
-        <f>IF(S9&gt;1,"✅ PASA",IF(S9&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X9" s="128">
-        <f>COUNTIF(T9:W9,"✅ PASA")+COUNTIF(T9:W9,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="W9" s="120" t="n"/>
+      <c r="X9" s="128" t="n"/>
       <c r="Y9" s="159" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z9" s="129">
-        <f>F9*0.93</f>
-        <v/>
-      </c>
-      <c r="AA9" s="129">
-        <f>F9*1.20</f>
-        <v/>
-      </c>
-      <c r="AB9" s="130" t="n"/>
-      <c r="AC9" s="131">
-        <f>IF(F9-Z9&lt;&gt;0,(AA9-F9)/MAX(F9-Z9,1),"-")</f>
-        <v/>
+          <t>👀 WATCHLIST #3</t>
+        </is>
+      </c>
+      <c r="Z9" s="129" t="n">
+        <v>609.5700000000001</v>
+      </c>
+      <c r="AA9" s="129" t="n">
+        <v>786.54</v>
+      </c>
+      <c r="AB9" s="130" t="n">
+        <v>473.2</v>
+      </c>
+      <c r="AC9" s="131" t="n">
+        <v>2.9</v>
       </c>
       <c r="AD9" s="132" t="inlineStr">
         <is>
-          <t>Semanal. Monitorear RS</t>
+          <t>Semanal. Alerta vol &gt;500K + breakout $740.91</t>
         </is>
       </c>
       <c r="AE9" s="160" t="inlineStr">
         <is>
-          <t>[1jun26] RS 82 — condicional. Activar cuando RS ≥ 85 → analizar con Claude.</t>
+          <t>[1jun26] RS 99. EPS +56.9%, ROE 33.8%, FCF 3.7%, D/E 0.01. F2 4/4. Vol 421K INSUFICIENTE (&lt;1M). Precio $655 (-11.5% de máx $740.91). Target analistas -27.8% (Wall St escéptico). Etapa 2. Trigger: vol &gt;500K + breakout $740.91.</t>
         </is>
       </c>
     </row>
@@ -1906,64 +1876,61 @@
       </c>
       <c r="B10" s="94" t="inlineStr">
         <is>
-          <t>VOXR</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="C10" s="95" t="inlineStr">
         <is>
-          <t>Vox Royalty Corp</t>
+          <t>The Vita Coco Company, Inc.</t>
         </is>
       </c>
       <c r="D10" s="95" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="E10" s="95" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F10" s="133" t="n">
-        <v>5.8</v>
+        <v>76.2</v>
       </c>
       <c r="G10" s="133" t="n">
-        <v>5.54</v>
+        <v>60.68</v>
       </c>
       <c r="H10" s="133" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="I10" s="95">
-        <f>IF(G10&gt;H10,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
+        <v>51.01</v>
+      </c>
+      <c r="I10" s="95" t="n"/>
       <c r="J10" s="96" t="n">
-        <v>49.831</v>
+        <v>0.614</v>
       </c>
       <c r="K10" s="95" t="n"/>
       <c r="L10" s="96" t="n">
-        <v>0.349</v>
+        <v>0.263</v>
       </c>
       <c r="M10" s="96" t="n">
-        <v>1.025</v>
+        <v>0.126</v>
       </c>
       <c r="N10" s="96" t="n">
-        <v>0.044</v>
+        <v>0.011</v>
       </c>
       <c r="O10" s="97" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="P10" s="98" t="n">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="Q10" s="96" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.958</v>
       </c>
       <c r="R10" s="96" t="n">
-        <v>0.332</v>
+        <v>-0.014</v>
       </c>
       <c r="S10" s="99" t="n">
-        <v>0.49</v>
+        <v>1.4</v>
       </c>
       <c r="T10" s="134" t="inlineStr">
         <is>
@@ -1977,43 +1944,36 @@
       </c>
       <c r="V10" s="95" t="inlineStr">
         <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W10" s="95">
-        <f>IF(S10&gt;1,"✅ PASA",IF(S10&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X10" s="100">
-        <f>COUNTIF(T10:W10,"✅ PASA")+COUNTIF(T10:W10,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="W10" s="95" t="n"/>
+      <c r="X10" s="100" t="n"/>
       <c r="Y10" s="157" t="inlineStr">
         <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z10" s="101">
-        <f>F10*0.93</f>
-        <v/>
-      </c>
-      <c r="AA10" s="101">
-        <f>F10*1.20</f>
-        <v/>
-      </c>
-      <c r="AB10" s="135" t="n"/>
-      <c r="AC10" s="102">
-        <f>IF(F10-Z10&lt;&gt;0,(AA10-F10)/MAX(F10-Z10,1),"-")</f>
-        <v/>
+          <t>👀 WATCHLIST #4</t>
+        </is>
+      </c>
+      <c r="Z10" s="101" t="n">
+        <v>70.87</v>
+      </c>
+      <c r="AA10" s="101" t="n">
+        <v>91.44</v>
+      </c>
+      <c r="AB10" s="135" t="n">
+        <v>75.11</v>
+      </c>
+      <c r="AC10" s="102" t="n">
+        <v>2.9</v>
       </c>
       <c r="AD10" s="136" t="inlineStr">
         <is>
-          <t>Mensual. Vigilar vol &gt;1M</t>
+          <t>Pullback SMA50 ~$60.68. Monitorear vol</t>
         </is>
       </c>
       <c r="AE10" s="158" t="inlineStr">
         <is>
-          <t>[30may26] Record Q1: net income $24.5M vs pérdida Q1 2025. GDXJ inclusion. Vol 513K (mitad del mínimo). RS 67. R/R 0.4x. Upside analistas insuficiente.</t>
+          <t>[1jun26] RS 93. EPS +61.4%, ROE 26.3%, FCF 1.1% (débil), D/E 0.04. F2 3/4. Precio $76.2 (+25.6% sobre SMA50 — sobreextendido). Vol -78.3% vs prom. Target analistas -1.4% (sin convicción). Etapa 2 tardía. Esperar pullback a SMA50 $60.68.</t>
         </is>
       </c>
     </row>
@@ -2023,114 +1983,104 @@
       </c>
       <c r="B11" s="121" t="inlineStr">
         <is>
-          <t>LPG</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="C11" s="120" t="inlineStr">
         <is>
-          <t>Dorian LPG Ltd</t>
+          <t>Aurinia Pharmaceuticals Inc.</t>
         </is>
       </c>
       <c r="D11" s="120" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="E11" s="120" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F11" s="122" t="n">
-        <v>40.33</v>
+        <v>15.31</v>
       </c>
       <c r="G11" s="122" t="n">
-        <v>37.12</v>
+        <v>15.52</v>
       </c>
       <c r="H11" s="122" t="n">
-        <v>30.01</v>
-      </c>
-      <c r="I11" s="120">
-        <f>IF(G11&gt;H11,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
+        <v>14.33</v>
+      </c>
+      <c r="I11" s="120" t="n"/>
       <c r="J11" s="123" t="n">
-        <v>9.012</v>
+        <v>0.472</v>
       </c>
       <c r="K11" s="120" t="n"/>
       <c r="L11" s="123" t="n">
-        <v>0.177</v>
+        <v>0.65</v>
       </c>
       <c r="M11" s="123" t="n">
-        <v>0.408</v>
+        <v>1</v>
       </c>
       <c r="N11" s="123" t="n">
-        <v>0.029</v>
+        <v>0.063</v>
       </c>
       <c r="O11" s="124" t="n">
-        <v>0.62</v>
+        <v>0.12</v>
       </c>
       <c r="P11" s="125" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="Q11" s="123" t="n">
-        <v>0.698</v>
+        <v>0.594</v>
       </c>
       <c r="R11" s="123" t="n">
-        <v>0.2</v>
+        <v>0.11</v>
       </c>
       <c r="S11" s="126" t="n">
-        <v>0.58</v>
+        <v>1.18</v>
       </c>
       <c r="T11" s="127" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="U11" s="120" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="V11" s="120" t="inlineStr">
         <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="W11" s="120">
-        <f>IF(S11&gt;1,"✅ PASA",IF(S11&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X11" s="128">
-        <f>COUNTIF(T11:W11,"✅ PASA")+COUNTIF(T11:W11,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="W11" s="120" t="n"/>
+      <c r="X11" s="128" t="n"/>
       <c r="Y11" s="159" t="inlineStr">
         <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z11" s="129">
-        <f>F11*0.93</f>
-        <v/>
-      </c>
-      <c r="AA11" s="129">
-        <f>F11*1.20</f>
-        <v/>
-      </c>
-      <c r="AB11" s="130" t="n"/>
-      <c r="AC11" s="131">
-        <f>IF(F11-Z11&lt;&gt;0,(AA11-F11)/MAX(F11-Z11,1),"-")</f>
-        <v/>
+          <t>👀 WATCHLIST</t>
+        </is>
+      </c>
+      <c r="Z11" s="129" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="AA11" s="129" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="AB11" s="130" t="n">
+        <v>17</v>
+      </c>
+      <c r="AC11" s="131" t="n">
+        <v>2.9</v>
       </c>
       <c r="AD11" s="132" t="inlineStr">
         <is>
-          <t>Sin revisión activa</t>
+          <t>Semanal. Activar cuando RS ≥ 85</t>
         </is>
       </c>
       <c r="AE11" s="160" t="inlineStr">
         <is>
-          <t>[30may26] Cíclico shipping. Q4 +102% pero Q1 -26.3% YoY. Revenue dependiente de tasas VLGC. F1 falla por revenue negativo en trimestre más reciente.</t>
+          <t>[1jun26] RS 81 — CONDICIONAL. EPS +47.2%, Sales 24.4% (❌&lt;25%), ROE 65%, FCF 6.3%, D/E 0.12. F3 1/3 (RS bajo). Precio $15.31 (-6.8% de máx $16.42). Activar cuando RS ≥ 85 → analizar con Claude.</t>
         </is>
       </c>
     </row>
@@ -2140,73 +2090,70 @@
       </c>
       <c r="B12" s="121" t="inlineStr">
         <is>
-          <t>FLXS</t>
+          <t>PAYS</t>
         </is>
       </c>
       <c r="C12" s="120" t="inlineStr">
         <is>
-          <t>Flexsteel Industries</t>
+          <t>Paysign, Inc.</t>
         </is>
       </c>
       <c r="D12" s="120" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E12" s="120" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F12" s="122" t="n">
-        <v>59.31</v>
+        <v>7.62</v>
       </c>
       <c r="G12" s="122" t="n">
-        <v>50.95</v>
+        <v>6.06</v>
       </c>
       <c r="H12" s="122" t="n">
-        <v>44.82</v>
-      </c>
-      <c r="I12" s="120">
-        <f>IF(G12&gt;H12,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
+        <v>5.19</v>
+      </c>
+      <c r="I12" s="120" t="n"/>
       <c r="J12" s="123" t="n">
-        <v>2.722</v>
+        <v>1.103</v>
       </c>
       <c r="K12" s="120" t="n"/>
       <c r="L12" s="123" t="n">
-        <v>0.181</v>
+        <v>0.221</v>
       </c>
       <c r="M12" s="123" t="n">
-        <v>0.068</v>
+        <v>0.114</v>
       </c>
       <c r="N12" s="123" t="n">
-        <v>0.09</v>
+        <v>0.021</v>
       </c>
       <c r="O12" s="124" t="n">
-        <v>0.29</v>
+        <v>0.11</v>
       </c>
       <c r="P12" s="125" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="Q12" s="123" t="n">
-        <v>0.704</v>
+        <v>0.473</v>
       </c>
       <c r="R12" s="123" t="n">
-        <v>0.189</v>
+        <v>0.306</v>
       </c>
       <c r="S12" s="126" t="n">
-        <v>0.049</v>
+        <v>0.948</v>
       </c>
       <c r="T12" s="127" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="U12" s="120" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="V12" s="120" t="inlineStr">
@@ -2214,1641 +2161,88 @@
           <t>2/3</t>
         </is>
       </c>
-      <c r="W12" s="120">
-        <f>IF(S12&gt;1,"✅ PASA",IF(S12&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X12" s="128">
-        <f>COUNTIF(T12:W12,"✅ PASA")+COUNTIF(T12:W12,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
+      <c r="W12" s="120" t="n"/>
+      <c r="X12" s="128" t="n"/>
       <c r="Y12" s="159" t="inlineStr">
         <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z12" s="129">
-        <f>F12*0.93</f>
-        <v/>
-      </c>
-      <c r="AA12" s="129">
-        <f>F12*1.20</f>
-        <v/>
-      </c>
-      <c r="AB12" s="130" t="n"/>
-      <c r="AC12" s="131">
-        <f>IF(F12-Z12&lt;&gt;0,(AA12-F12)/MAX(F12-Z12,1),"-")</f>
-        <v/>
+          <t>👀 WATCHLIST</t>
+        </is>
+      </c>
+      <c r="Z12" s="129" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="AA12" s="129" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="AB12" s="130" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="AC12" s="131" t="n">
+        <v>2.9</v>
       </c>
       <c r="AD12" s="132" t="inlineStr">
         <is>
-          <t>Sin revisión activa</t>
+          <t>Semanal. Activar cuando RS ≥ 85 + vol promedio &gt;1M</t>
         </is>
       </c>
       <c r="AE12" s="160" t="inlineStr">
         <is>
-          <t>[30may26] Revenue Q3 +1% YoY, Q2 +9% YoY. Muy lejos del umbral 25%. Volumen 48K irrisorio. Manufactura muebles sin catalizador. F1 falla.</t>
+          <t>[1jun26] RS 71 — CONDICIONAL. EPS +110.3%, ROE 22.1%, FCF 2.1%, D/E 0.11. F2 4/4. Vol 948K (&lt;1M). Precio $7.62 (-11% de máx $8.56). Activar cuando RS ≥ 85 Y vol promedio &gt; 1M. Trigger: breakout $8.56.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" s="72">
-      <c r="A13" s="120" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="121" t="inlineStr">
-        <is>
-          <t>NVGS</t>
-        </is>
-      </c>
-      <c r="C13" s="120" t="inlineStr">
-        <is>
-          <t>Navigator Holdings</t>
-        </is>
-      </c>
-      <c r="D13" s="120" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="E13" s="120" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F13" s="122" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="G13" s="122" t="n">
-        <v>21.17</v>
-      </c>
-      <c r="H13" s="122" t="n">
-        <v>18.22</v>
-      </c>
-      <c r="I13" s="120">
-        <f>IF(G13&gt;H13,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J13" s="123" t="n">
-        <v>0.312</v>
-      </c>
+      <c r="A13" s="120" t="inlineStr">
+        <is>
+          <t>📌 LEYENDA  |  🔵 Azul = INPUTS manuales  |  ⚫ Negro = Fórmulas  |  🟢 OPERAR ≥3.5/4  |  🟡 WATCHLIST 2.5–3/4  |  🔴 NO OPERAR &lt;2.5  |  🚫 DESCARTAR: Falla F1</t>
+        </is>
+      </c>
+      <c r="B13" s="121" t="n"/>
+      <c r="C13" s="120" t="n"/>
+      <c r="D13" s="120" t="n"/>
+      <c r="E13" s="120" t="n"/>
+      <c r="F13" s="122" t="n"/>
+      <c r="G13" s="122" t="n"/>
+      <c r="H13" s="122" t="n"/>
+      <c r="I13" s="120" t="n"/>
+      <c r="J13" s="123" t="n"/>
       <c r="K13" s="120" t="n"/>
-      <c r="L13" s="123" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="M13" s="123" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="N13" s="123" t="n">
-        <v>0.092</v>
-      </c>
-      <c r="O13" s="124" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="P13" s="125" t="n">
-        <v>61</v>
-      </c>
-      <c r="Q13" s="123" t="n">
-        <v>0.414</v>
-      </c>
-      <c r="R13" s="123" t="n">
-        <v>0.164</v>
-      </c>
-      <c r="S13" s="126" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="T13" s="127" t="inlineStr">
-        <is>
-          <t>🚫</t>
-        </is>
-      </c>
-      <c r="U13" s="120" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V13" s="120" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W13" s="120">
-        <f>IF(S13&gt;1,"✅ PASA",IF(S13&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X13" s="128">
-        <f>COUNTIF(T13:W13,"✅ PASA")+COUNTIF(T13:W13,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y13" s="159" t="inlineStr">
-        <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z13" s="129">
-        <f>F13*0.93</f>
-        <v/>
-      </c>
-      <c r="AA13" s="129">
-        <f>F13*1.20</f>
-        <v/>
-      </c>
+      <c r="L13" s="123" t="n"/>
+      <c r="M13" s="123" t="n"/>
+      <c r="N13" s="123" t="n"/>
+      <c r="O13" s="124" t="n"/>
+      <c r="P13" s="125" t="n"/>
+      <c r="Q13" s="123" t="n"/>
+      <c r="R13" s="123" t="n"/>
+      <c r="S13" s="126" t="n"/>
+      <c r="T13" s="127" t="n"/>
+      <c r="U13" s="120" t="n"/>
+      <c r="V13" s="120" t="n"/>
+      <c r="W13" s="120" t="n"/>
+      <c r="X13" s="128" t="n"/>
+      <c r="Y13" s="159" t="n"/>
+      <c r="Z13" s="129" t="n"/>
+      <c r="AA13" s="129" t="n"/>
       <c r="AB13" s="130" t="n"/>
-      <c r="AC13" s="131">
-        <f>IF(F13-Z13&lt;&gt;0,(AA13-F13)/MAX(F13-Z13,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD13" s="132" t="inlineStr">
-        <is>
-          <t>Sin revisión activa</t>
-        </is>
-      </c>
-      <c r="AE13" s="160" t="inlineStr">
-        <is>
-          <t>[30may26] Revenue Q1 $121M vs estimado $151M — miss $30M. Cíclico shipping gas. Record net income por venta activos (one-time $15.2M). F1 falla.</t>
-        </is>
-      </c>
+      <c r="AC13" s="131" t="n"/>
+      <c r="AD13" s="132" t="n"/>
+      <c r="AE13" s="160" t="n"/>
     </row>
-    <row r="14" ht="42" customHeight="1" s="72">
-      <c r="A14" s="120" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="121" t="inlineStr">
-        <is>
-          <t>SPIR</t>
-        </is>
-      </c>
-      <c r="C14" s="120" t="inlineStr">
-        <is>
-          <t>Spire Global</t>
-        </is>
-      </c>
-      <c r="D14" s="120" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="E14" s="120" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F14" s="122" t="n">
-        <v>22.71</v>
-      </c>
-      <c r="G14" s="122" t="n">
-        <v>17.75</v>
-      </c>
-      <c r="H14" s="122" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="I14" s="120">
-        <f>IF(G14&gt;H14,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J14" s="123" t="n">
-        <v>0.464</v>
-      </c>
-      <c r="K14" s="120" t="n"/>
-      <c r="L14" s="123" t="n">
-        <v>1.012</v>
-      </c>
-      <c r="M14" s="123" t="n">
-        <v>0.771</v>
-      </c>
-      <c r="N14" s="123" t="n">
-        <v>0.011</v>
-      </c>
-      <c r="O14" s="124" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="P14" s="125" t="n">
-        <v>91</v>
-      </c>
-      <c r="Q14" s="123" t="n">
-        <v>0.382</v>
-      </c>
-      <c r="R14" s="123" t="n">
-        <v>-0.103</v>
-      </c>
-      <c r="S14" s="126" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="T14" s="127" t="inlineStr">
-        <is>
-          <t>🚫</t>
-        </is>
-      </c>
-      <c r="U14" s="120" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V14" s="120" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W14" s="120">
-        <f>IF(S14&gt;1,"✅ PASA",IF(S14&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X14" s="128">
-        <f>COUNTIF(T14:W14,"✅ PASA")+COUNTIF(T14:W14,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y14" s="159" t="inlineStr">
-        <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z14" s="129">
-        <f>F14*0.93</f>
-        <v/>
-      </c>
-      <c r="AA14" s="129">
-        <f>F14*1.20</f>
-        <v/>
-      </c>
-      <c r="AB14" s="130" t="n"/>
-      <c r="AC14" s="131">
-        <f>IF(F14-Z14&lt;&gt;0,(AA14-F14)/MAX(F14-Z14,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD14" s="132" t="inlineStr">
-        <is>
-          <t>Sin revisión activa</t>
-        </is>
-      </c>
-      <c r="AE14" s="160" t="inlineStr">
-        <is>
-          <t>[30may26] Revenue Q1 $15.8M vs estimado $38.1M — miss brutal -58%. Revenue core -26.9% YoY. Negocio en restructuración. F1 falla sin discusión.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1" s="72">
-      <c r="A15" s="120" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="121" t="inlineStr">
-        <is>
-          <t>TRS</t>
-        </is>
-      </c>
-      <c r="C15" s="120" t="inlineStr">
-        <is>
-          <t>TriMas Corporation</t>
-        </is>
-      </c>
-      <c r="D15" s="120" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="E15" s="120" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F15" s="122" t="n">
-        <v>41</v>
-      </c>
-      <c r="G15" s="122" t="n">
-        <v>38.13</v>
-      </c>
-      <c r="H15" s="122" t="n">
-        <v>36.53</v>
-      </c>
-      <c r="I15" s="120">
-        <f>IF(G15&gt;H15,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J15" s="123" t="n">
-        <v>63.479</v>
-      </c>
-      <c r="K15" s="120" t="n"/>
-      <c r="L15" s="123" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="M15" s="123" t="n">
-        <v>1.373</v>
-      </c>
-      <c r="N15" s="123" t="n">
-        <v>0.234</v>
-      </c>
-      <c r="O15" s="124" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="P15" s="125" t="n">
-        <v>62</v>
-      </c>
-      <c r="Q15" s="123" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="R15" s="123" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="S15" s="126" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T15" s="127" t="inlineStr">
-        <is>
-          <t>🚫</t>
-        </is>
-      </c>
-      <c r="U15" s="120" t="inlineStr">
-        <is>
-          <t>1/4</t>
-        </is>
-      </c>
-      <c r="V15" s="120" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W15" s="120">
-        <f>IF(S15&gt;1,"✅ PASA",IF(S15&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X15" s="128">
-        <f>COUNTIF(T15:W15,"✅ PASA")+COUNTIF(T15:W15,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y15" s="159" t="inlineStr">
-        <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z15" s="129">
-        <f>F15*0.93</f>
-        <v/>
-      </c>
-      <c r="AA15" s="129">
-        <f>F15*1.20</f>
-        <v/>
-      </c>
-      <c r="AB15" s="130" t="n"/>
-      <c r="AC15" s="131">
-        <f>IF(F15-Z15&lt;&gt;0,(AA15-F15)/MAX(F15-Z15,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD15" s="132" t="inlineStr">
-        <is>
-          <t>Sin revisión activa</t>
-        </is>
-      </c>
-      <c r="AE15" s="160" t="inlineStr">
-        <is>
-          <t>[30may26] ROE 1.7% elimina F2 inmediatamente. Sin momentum de analistas. Sin catalizador visible. F2 falla 2/4 como mínimo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1" s="72">
-      <c r="A16" s="120" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="121" t="inlineStr">
-        <is>
-          <t>CTS</t>
-        </is>
-      </c>
-      <c r="C16" s="120" t="inlineStr">
-        <is>
-          <t>CTS Corporation</t>
-        </is>
-      </c>
-      <c r="D16" s="120" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="E16" s="120" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F16" s="122" t="n">
-        <v>64.43000000000001</v>
-      </c>
-      <c r="G16" s="122" t="n">
-        <v>55.37</v>
-      </c>
-      <c r="H16" s="122" t="n">
-        <v>47.44</v>
-      </c>
-      <c r="I16" s="120">
-        <f>IF(G16&gt;H16,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J16" s="123" t="n">
-        <v>0.287</v>
-      </c>
-      <c r="K16" s="120" t="n"/>
-      <c r="L16" s="123" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="M16" s="123" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="N16" s="123" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="O16" s="124" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="P16" s="125" t="n">
-        <v>64</v>
-      </c>
-      <c r="Q16" s="123" t="n">
-        <v>0.991</v>
-      </c>
-      <c r="R16" s="123" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="S16" s="126" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="T16" s="127" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U16" s="120" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V16" s="120" t="inlineStr">
-        <is>
-          <t>0/3</t>
-        </is>
-      </c>
-      <c r="W16" s="120">
-        <f>IF(S16&gt;1,"✅ PASA",IF(S16&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X16" s="128">
-        <f>COUNTIF(T16:W16,"✅ PASA")+COUNTIF(T16:W16,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y16" s="159" t="inlineStr">
-        <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z16" s="129">
-        <f>F16*0.93</f>
-        <v/>
-      </c>
-      <c r="AA16" s="129">
-        <f>F16*1.20</f>
-        <v/>
-      </c>
-      <c r="AB16" s="130" t="n"/>
-      <c r="AC16" s="131">
-        <f>IF(F16-Z16&lt;&gt;0,(AA16-F16)/MAX(F16-Z16,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD16" s="132" t="inlineStr">
-        <is>
-          <t>Sin revisión activa</t>
-        </is>
-      </c>
-      <c r="AE16" s="160" t="inlineStr">
-        <is>
-          <t>[30may26] Analistas ven downside -10% desde precio actual. Upside negativo destruye F3 completamente. F3 0/3. Sin momentum institucional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1" s="72">
-      <c r="A17" s="161" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="162" t="inlineStr">
-        <is>
-          <t>ABUS</t>
-        </is>
-      </c>
-      <c r="C17" s="161" t="inlineStr">
-        <is>
-          <t>Arbutus Biopharma</t>
-        </is>
-      </c>
-      <c r="D17" s="161" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="E17" s="161" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F17" s="163" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="G17" s="163" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="H17" s="163" t="n">
-        <v>4.36</v>
-      </c>
-      <c r="I17" s="164">
-        <f>IF(G17&gt;H17,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J17" s="165" t="n">
-        <v>7.919</v>
-      </c>
-      <c r="K17" s="161" t="n"/>
-      <c r="L17" s="165" t="n">
-        <v>0.947</v>
-      </c>
-      <c r="M17" s="165" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="N17" s="165" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="O17" s="166" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P17" s="161" t="n">
-        <v>52</v>
-      </c>
-      <c r="Q17" s="165" t="n">
-        <v>0.719</v>
-      </c>
-      <c r="R17" s="165" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="S17" s="161" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="T17" s="167" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U17" s="164" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="V17" s="164" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W17" s="164">
-        <f>IF(S17&gt;1,"✅ PASA",IF(S17&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X17" s="164">
-        <f>COUNTIF(T17:W17,"✅ PASA")+COUNTIF(T17:W17,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y17" s="168" t="inlineStr">
-        <is>
-          <t>🚫 ELIMINADO</t>
-        </is>
-      </c>
-      <c r="Z17" s="164">
-        <f>F17*0.93</f>
-        <v/>
-      </c>
-      <c r="AA17" s="164">
-        <f>F17*1.20</f>
-        <v/>
-      </c>
-      <c r="AB17" s="169" t="n"/>
-      <c r="AC17" s="164">
-        <f>IF(F17-Z17&lt;&gt;0,(AA17-F17)/MAX(F17-Z17,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD17" s="169" t="inlineStr">
-        <is>
-          <t>Sin revisión — biotech</t>
-        </is>
-      </c>
-      <c r="AE17" s="170" t="inlineStr">
-        <is>
-          <t>[30may26] BIOTECH EXCLUIDO del universo CAN SLIM. Sin producto comercializado con revenue recurrente real. FCF negativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1" s="72">
-      <c r="A18" s="95" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="94" t="inlineStr">
-        <is>
-          <t>ABX</t>
-        </is>
-      </c>
-      <c r="C18" s="95" t="inlineStr">
-        <is>
-          <t>Abacus Global Mgmt</t>
-        </is>
-      </c>
-      <c r="D18" s="95" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
-      <c r="E18" s="95" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F18" s="133" t="n">
-        <v>8.98</v>
-      </c>
-      <c r="G18" s="133" t="n">
-        <v>8.94</v>
-      </c>
-      <c r="H18" s="133" t="n">
-        <v>7.62</v>
-      </c>
-      <c r="I18" s="103">
-        <f>IF(G18&gt;H18,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J18" s="96" t="n">
-        <v>0.5659999999999999</v>
-      </c>
-      <c r="K18" s="95" t="n"/>
-      <c r="L18" s="96" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="M18" s="96" t="n">
-        <v>0.156</v>
-      </c>
-      <c r="N18" s="96" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="O18" s="97" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="P18" s="95" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q18" s="96" t="n">
-        <v>0.285</v>
-      </c>
-      <c r="R18" s="96" t="n">
-        <v>0.513</v>
-      </c>
-      <c r="S18" s="95" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="T18" s="152" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U18" s="103" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V18" s="103" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W18" s="103">
-        <f>IF(S18&gt;1,"✅ PASA",IF(S18&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X18" s="103">
-        <f>COUNTIF(T18:W18,"✅ PASA")+COUNTIF(T18:W18,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y18" s="171" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z18" s="103">
-        <f>F18*0.93</f>
-        <v/>
-      </c>
-      <c r="AA18" s="103">
-        <f>F18*1.20</f>
-        <v/>
-      </c>
-      <c r="AB18" s="153" t="n"/>
-      <c r="AC18" s="103">
-        <f>IF(F18-Z18&lt;&gt;0,(AA18-F18)/MAX(F18-Z18,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD18" s="153" t="inlineStr">
-        <is>
-          <t>Mensual. Vigilar inst. &gt;40%</t>
-        </is>
-      </c>
-      <c r="AE18" s="158" t="inlineStr">
-        <is>
-          <t>[30may26] Revenue +35% YoY. Net income +59%. OCF swing $91.7M. ROIC 17%, EBITDA margin 55%. FRENO: Inst. 28.5% bajo umbral. Upside +15% insuficiente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1" s="72">
-      <c r="A19" s="161" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" s="162" t="inlineStr">
-        <is>
-          <t>GTY</t>
-        </is>
-      </c>
-      <c r="C19" s="161" t="inlineStr">
-        <is>
-          <t>Getty Realty Corp</t>
-        </is>
-      </c>
-      <c r="D19" s="161" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="E19" s="161" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F19" s="163" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="G19" s="163" t="n">
-        <v>32.97</v>
-      </c>
-      <c r="H19" s="163" t="n">
-        <v>29.31</v>
-      </c>
-      <c r="I19" s="164">
-        <f>IF(G19&gt;H19,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J19" s="165" t="n">
-        <v>0.801</v>
-      </c>
-      <c r="K19" s="161" t="n"/>
-      <c r="L19" s="165" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="M19" s="165" t="n">
-        <v>0.401</v>
-      </c>
-      <c r="N19" s="165" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="O19" s="166" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="P19" s="161" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q19" s="165" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-      <c r="R19" s="165" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="S19" s="161" t="n"/>
-      <c r="T19" s="167" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U19" s="164" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="V19" s="164" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W19" s="164">
-        <f>IF(S19&gt;1,"✅ PASA",IF(S19&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X19" s="164">
-        <f>COUNTIF(T19:W19,"✅ PASA")+COUNTIF(T19:W19,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y19" s="168" t="inlineStr">
-        <is>
-          <t>🚫 ELIMINADO</t>
-        </is>
-      </c>
-      <c r="Z19" s="164">
-        <f>F19*0.93</f>
-        <v/>
-      </c>
-      <c r="AA19" s="164">
-        <f>F19*1.20</f>
-        <v/>
-      </c>
-      <c r="AB19" s="169" t="n"/>
-      <c r="AC19" s="164">
-        <f>IF(F19-Z19&lt;&gt;0,(AA19-F19)/MAX(F19-Z19,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD19" s="169" t="inlineStr">
-        <is>
-          <t>Sin revisión — REIT</t>
-        </is>
-      </c>
-      <c r="AE19" s="170" t="inlineStr">
-        <is>
-          <t>[30may26] REIT — estructura incompatible con CAN SLIM. Upside analistas solo 6.7%. Dividendo alto pero no aplica metodología de crecimiento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="42" customHeight="1" s="72">
-      <c r="A20" s="95" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" s="94" t="inlineStr">
-        <is>
-          <t>DDI</t>
-        </is>
-      </c>
-      <c r="C20" s="95" t="inlineStr">
-        <is>
-          <t>DoubleDown Interactive</t>
-        </is>
-      </c>
-      <c r="D20" s="95" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="E20" s="95" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F20" s="133" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="G20" s="133" t="n">
-        <v>10.03</v>
-      </c>
-      <c r="H20" s="133" t="n">
-        <v>9.27</v>
-      </c>
-      <c r="I20" s="103">
-        <f>IF(G20&gt;H20,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J20" s="96" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="K20" s="95" t="n"/>
-      <c r="L20" s="96" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="M20" s="96" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="N20" s="96" t="n">
-        <v>0.177</v>
-      </c>
-      <c r="O20" s="97" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="P20" s="95" t="n">
-        <v>43</v>
-      </c>
-      <c r="Q20" s="96" t="n">
-        <v>0.207</v>
-      </c>
-      <c r="R20" s="96" t="n">
-        <v>0.406</v>
-      </c>
-      <c r="S20" s="95" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="T20" s="152" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U20" s="103" t="inlineStr">
-        <is>
-          <t>4/4</t>
-        </is>
-      </c>
-      <c r="V20" s="103" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W20" s="103">
-        <f>IF(S20&gt;1,"✅ PASA",IF(S20&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X20" s="103">
-        <f>COUNTIF(T20:W20,"✅ PASA")+COUNTIF(T20:W20,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y20" s="171" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z20" s="103">
-        <f>F20*0.93</f>
-        <v/>
-      </c>
-      <c r="AA20" s="103">
-        <f>F20*1.20</f>
-        <v/>
-      </c>
-      <c r="AB20" s="153" t="n"/>
-      <c r="AC20" s="103">
-        <f>IF(F20-Z20&lt;&gt;0,(AA20-F20)/MAX(F20-Z20,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD20" s="153" t="inlineStr">
-        <is>
-          <t>Mensual. Monitorear takeover</t>
-        </is>
-      </c>
-      <c r="AE20" s="158" t="inlineStr">
-        <is>
-          <t>[30may26] EPS +48% YoY. $500M net cash. P/E 4x bajo. RIESGO CRÍTICO: oferta no vinculante de adquisición por accionista controlador (squeeze-out minoritarios). Vol 123K ilíquido.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="42" customHeight="1" s="72">
-      <c r="A21" s="120" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="121" t="inlineStr">
-        <is>
-          <t>PLGO</t>
-        </is>
-      </c>
-      <c r="C21" s="120" t="inlineStr">
-        <is>
-          <t>PLGO Insurance</t>
-        </is>
-      </c>
-      <c r="D21" s="120" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
-      <c r="E21" s="120" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F21" s="122" t="n">
-        <v>21.58</v>
-      </c>
-      <c r="G21" s="122" t="n">
-        <v>20.71</v>
-      </c>
-      <c r="H21" s="122" t="n">
-        <v>18.97</v>
-      </c>
-      <c r="I21" s="154">
-        <f>IF(G21&gt;H21,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J21" s="123" t="n">
-        <v>3.541</v>
-      </c>
-      <c r="K21" s="120" t="n"/>
-      <c r="L21" s="123" t="n">
-        <v>0.162</v>
-      </c>
-      <c r="M21" s="123" t="n">
-        <v>0.153</v>
-      </c>
-      <c r="N21" s="123" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="O21" s="124" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="P21" s="120" t="n">
-        <v>47</v>
-      </c>
-      <c r="Q21" s="123" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-      <c r="R21" s="123" t="n">
-        <v>0.107</v>
-      </c>
-      <c r="S21" s="120" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="T21" s="154" t="inlineStr">
-        <is>
-          <t>🚫</t>
-        </is>
-      </c>
-      <c r="U21" s="154" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V21" s="154" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="W21" s="154">
-        <f>IF(S21&gt;1,"✅ PASA",IF(S21&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X21" s="154">
-        <f>COUNTIF(T21:W21,"✅ PASA")+COUNTIF(T21:W21,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y21" s="172" t="inlineStr">
-        <is>
-          <t>🚫 DESCARTAR</t>
-        </is>
-      </c>
-      <c r="Z21" s="154">
-        <f>F21*0.93</f>
-        <v/>
-      </c>
-      <c r="AA21" s="154">
-        <f>F21*1.20</f>
-        <v/>
-      </c>
-      <c r="AB21" s="156" t="n"/>
-      <c r="AC21" s="154">
-        <f>IF(F21-Z21&lt;&gt;0,(AA21-F21)/MAX(F21-Z21,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD21" s="156" t="inlineStr">
-        <is>
-          <t>Sin revisión activa</t>
-        </is>
-      </c>
-      <c r="AE21" s="160" t="inlineStr">
-        <is>
-          <t>[30may26] Revenue Q1 -7.3% YoY. 4 revisiones EPS a la baja vs 1 al alza. Recuperación underwriting (combined ratio 115%→86%) no es crecimiento. F1 falla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="42" customHeight="1" s="72">
-      <c r="A22" s="95" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="94" t="inlineStr">
-        <is>
-          <t>OPRA</t>
-        </is>
-      </c>
-      <c r="C22" s="95" t="inlineStr">
-        <is>
-          <t>Opera Limited</t>
-        </is>
-      </c>
-      <c r="D22" s="95" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="E22" s="95" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="F22" s="133" t="n">
-        <v>18.78</v>
-      </c>
-      <c r="G22" s="133" t="n">
-        <v>16.63</v>
-      </c>
-      <c r="H22" s="133" t="n">
-        <v>15.3</v>
-      </c>
-      <c r="I22" s="103">
-        <f>IF(G22&gt;H22,"✅ ALCISTA","❌ BAJISTA")</f>
-        <v/>
-      </c>
-      <c r="J22" s="96" t="n">
-        <v>0.356</v>
-      </c>
-      <c r="K22" s="95" t="n"/>
-      <c r="L22" s="96" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="M22" s="96" t="n">
-        <v>0.177</v>
-      </c>
-      <c r="N22" s="96" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="O22" s="97" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="P22" s="95" t="n">
-        <v>38</v>
-      </c>
-      <c r="Q22" s="96" t="n">
-        <v>0.168</v>
-      </c>
-      <c r="R22" s="96" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S22" s="95" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="T22" s="103" t="inlineStr">
-        <is>
-          <t>⚠️</t>
-        </is>
-      </c>
-      <c r="U22" s="103" t="inlineStr">
-        <is>
-          <t>4/4</t>
-        </is>
-      </c>
-      <c r="V22" s="103" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="W22" s="103">
-        <f>IF(S22&gt;1,"✅ PASA",IF(S22&gt;0.5,"⚠ PARCIAL","❌ FALLA"))</f>
-        <v/>
-      </c>
-      <c r="X22" s="103">
-        <f>COUNTIF(T22:W22,"✅ PASA")+COUNTIF(T22:W22,"⚠ PARCIAL")*0.5</f>
-        <v/>
-      </c>
-      <c r="Y22" s="171" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="Z22" s="103">
-        <f>F22*0.93</f>
-        <v/>
-      </c>
-      <c r="AA22" s="103">
-        <f>F22*1.20</f>
-        <v/>
-      </c>
-      <c r="AB22" s="153" t="n"/>
-      <c r="AC22" s="103">
-        <f>IF(F22-Z22&lt;&gt;0,(AA22-F22)/MAX(F22-Z22,1),"-")</f>
-        <v/>
-      </c>
-      <c r="AD22" s="153" t="inlineStr">
-        <is>
-          <t>Q2 jul26. Vigilar rev &gt;25%</t>
-        </is>
-      </c>
-      <c r="AE22" s="158" t="inlineStr">
-        <is>
-          <t>[30may26] Revenue +23% borderline (2pts bajo umbral). EPS +54% beat. 20T Rule of 40. Inst. 16.8% muy bajo. Guidance FY26 raised $727-740M. Cayman/Oslo descuento estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="72">
-      <c r="A23" s="0" t="n">
-        <v>17</v>
-      </c>
-      <c r="B23" s="0" t="inlineStr">
-        <is>
-          <t>VISN</t>
-        </is>
-      </c>
-      <c r="C23" s="0" t="inlineStr">
-        <is>
-          <t>Vistance Networks, Inc.</t>
-        </is>
-      </c>
-      <c r="D23" s="0" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="E23" s="0" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>12.39</v>
-      </c>
-      <c r="G23" t="n">
-        <v>10.42</v>
-      </c>
-      <c r="H23" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.131</v>
-      </c>
-      <c r="M23" t="n">
-        <v>3.477</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="P23" s="0" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.372</v>
-      </c>
-      <c r="S23" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="T23" s="0" t="inlineStr">
-        <is>
-          <t>⚠️</t>
-        </is>
-      </c>
-      <c r="U23" s="0" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V23" s="0" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="W23" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X23" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y23" s="0" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST #1</t>
-        </is>
-      </c>
-      <c r="AD23" s="0" t="inlineStr">
-        <is>
-          <t>Diario. Alerta ruptura $12.80 vol≥10.6M</t>
-        </is>
-      </c>
-      <c r="AE23" s="0" t="inlineStr">
-        <is>
-          <t>[1jun26] RS 99. EPS +602.6% YoY, Sales +21.6% (❌&lt;25%), ROE 13.1% (❌&lt;17%), FCF 27%, D/E 0.01. F3 3/3 (único). Precio $12.39 (-3.2% de máx $12.80). Vol -59.1% — sin breakout. Etapa 2 tardía, riesgo Etapa 3. Trigger: ruptura $12.80 con vol ≥ 10.6M.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1" s="72">
-      <c r="A24" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="B24" s="0" t="inlineStr">
-        <is>
-          <t>YOU</t>
-        </is>
-      </c>
-      <c r="C24" s="0" t="inlineStr">
-        <is>
-          <t>Clear Secure, Inc.</t>
-        </is>
-      </c>
-      <c r="D24" s="0" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="E24" s="0" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="F24" s="0" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="G24" s="0" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="H24" s="0" t="n">
-        <v>40.34</v>
-      </c>
-      <c r="L24" s="0" t="n">
-        <v>1.095</v>
-      </c>
-      <c r="M24" s="0" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="N24" s="0" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="O24" s="0" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="P24" s="0" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q24" s="0" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="R24" s="0" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="S24" s="0" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="T24" s="0" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U24" s="0" t="inlineStr">
-        <is>
-          <t>4/4</t>
-        </is>
-      </c>
-      <c r="V24" s="0" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="W24" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X24" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y24" s="0" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST #2</t>
-        </is>
-      </c>
-      <c r="AD24" s="0" t="inlineStr">
-        <is>
-          <t>Diario. Alerta breakout $62.36 vol≥50%</t>
-        </is>
-      </c>
-      <c r="AE24" s="0" t="inlineStr">
-        <is>
-          <t>[1jun26] RS 99. EPS +52.7% YoY, ROE 109.5%, FCF 4.5%, D/E 0.52. Precio $57.1 (-8.4% de máx $62.36). Vol -65% vs prom — sin breakout. Etapa 2. Esperar vol ≥50% sobre prom 50d en quiebre de $62.36.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="72">
-      <c r="A25" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="B25" s="0" t="inlineStr">
-        <is>
-          <t>AGX</t>
-        </is>
-      </c>
-      <c r="C25" s="0" t="inlineStr">
-        <is>
-          <t>Argan, Inc.</t>
-        </is>
-      </c>
-      <c r="D25" s="0" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="E25" s="0" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="F25" s="0" t="n">
-        <v>655.45</v>
-      </c>
-      <c r="G25" s="0" t="n">
-        <v>621.51</v>
-      </c>
-      <c r="H25" s="0" t="n">
-        <v>400.54</v>
-      </c>
-      <c r="L25" s="0" t="n">
-        <v>0.338</v>
-      </c>
-      <c r="M25" s="0" t="n">
-        <v>0.146</v>
-      </c>
-      <c r="N25" s="0" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="O25" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="P25" s="0" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q25" s="0" t="n">
-        <v>1.018</v>
-      </c>
-      <c r="R25" s="0" t="n">
-        <v>-0.278</v>
-      </c>
-      <c r="S25" s="0" t="n">
-        <v>0.421</v>
-      </c>
-      <c r="T25" s="0" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U25" s="0" t="inlineStr">
-        <is>
-          <t>4/4</t>
-        </is>
-      </c>
-      <c r="V25" s="0" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="W25" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X25" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y25" s="0" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST #3</t>
-        </is>
-      </c>
-      <c r="AD25" s="0" t="inlineStr">
-        <is>
-          <t>Semanal. Alerta vol &gt;500K + breakout $740.91</t>
-        </is>
-      </c>
-      <c r="AE25" s="0" t="inlineStr">
-        <is>
-          <t>[1jun26] RS 99. EPS +56.9% YoY, ROE 33.8%, FCF 3.7%, D/E 0.01. Vol 421K INSUFICIENTE (&lt;1M). Precio $655 (-11.5% de máx $740.91). Target analistas -27.8% (Wall St escéptico). Etapa 2. Trigger: vol &gt;500K + breakout $740.91.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="72">
-      <c r="A26" s="0" t="n">
-        <v>20</v>
-      </c>
-      <c r="B26" s="0" t="inlineStr">
-        <is>
-          <t>COCO</t>
-        </is>
-      </c>
-      <c r="C26" s="0" t="inlineStr">
-        <is>
-          <t>The Vita Coco Company, Inc.</t>
-        </is>
-      </c>
-      <c r="D26" s="0" t="inlineStr">
-        <is>
-          <t>Consumer Defensive</t>
-        </is>
-      </c>
-      <c r="E26" s="0" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="F26" s="0" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="G26" s="0" t="n">
-        <v>60.68</v>
-      </c>
-      <c r="H26" s="0" t="n">
-        <v>51.01</v>
-      </c>
-      <c r="L26" s="0" t="n">
-        <v>0.263</v>
-      </c>
-      <c r="M26" s="0" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="N26" s="0" t="n">
-        <v>0.011</v>
-      </c>
-      <c r="O26" s="0" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="P26" s="0" t="n">
-        <v>93</v>
-      </c>
-      <c r="Q26" s="0" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="R26" s="0" t="n">
-        <v>-0.014</v>
-      </c>
-      <c r="S26" s="0" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="T26" s="0" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="U26" s="0" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
-      <c r="V26" s="0" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="W26" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X26" s="0" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y26" s="0" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST #4</t>
-        </is>
-      </c>
-      <c r="AD26" s="0" t="inlineStr">
-        <is>
-          <t>Pullback SMA50 ~$60.68. Monitorear vol</t>
-        </is>
-      </c>
-      <c r="AE26" s="0" t="inlineStr">
-        <is>
-          <t>[1jun26] RS 93. EPS +61.4% YoY, ROE 26.3%, FCF 1.1% (débil), D/E 0.04. Precio $76.2 (+25.6% sobre SMA50 — sobreextendido). Vol -78.3% vs prom. Target analistas -1.4% (sin convicción). Etapa 2 tardía. Esperar pullback a SMA50 $60.68.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="72">
-      <c r="A27" s="95" t="n"/>
-      <c r="B27" s="94" t="n"/>
-      <c r="C27" s="95" t="n"/>
-      <c r="D27" s="95" t="n"/>
-      <c r="E27" s="95" t="n"/>
-      <c r="F27" s="84" t="n"/>
-      <c r="G27" s="84" t="n"/>
-      <c r="H27" s="84" t="n"/>
-      <c r="I27" s="103" t="n"/>
-      <c r="J27" s="96" t="n"/>
-      <c r="K27" s="95" t="n"/>
-      <c r="L27" s="96" t="n"/>
-      <c r="M27" s="96" t="n"/>
-      <c r="N27" s="96" t="n"/>
-      <c r="O27" s="97" t="n"/>
-      <c r="P27" s="95" t="n"/>
-      <c r="Q27" s="96" t="n"/>
-      <c r="R27" s="96" t="n"/>
-      <c r="S27" s="95" t="n"/>
-      <c r="T27" s="103" t="n"/>
-      <c r="U27" s="103" t="n"/>
-      <c r="V27" s="103" t="n"/>
-      <c r="W27" s="103" t="n"/>
-      <c r="X27" s="103" t="n"/>
-      <c r="Y27" s="103" t="n"/>
-      <c r="Z27" s="103" t="n"/>
-      <c r="AA27" s="103" t="n"/>
-      <c r="AC27" s="103" t="n"/>
-      <c r="AE27" s="95" t="n"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="72">
-      <c r="A28" s="114" t="inlineStr">
-        <is>
-          <t>📌 LEYENDA  |  🔵 Azul = INPUTS manuales  |  ⚫ Negro = Fórmulas  |  🟢 OPERAR ≥3.5/4  |  🟡 WATCHLIST 2.5–3/4  |  🔴 NO OPERAR &lt;2.5  |  🚫 DESCARTAR: Falla F1</t>
-        </is>
-      </c>
-    </row>
+    <row r="14" ht="42" customHeight="1" s="72"/>
+    <row r="15" ht="42" customHeight="1" s="72"/>
+    <row r="16" ht="42" customHeight="1" s="72"/>
+    <row r="17" ht="42" customHeight="1" s="72"/>
+    <row r="18" ht="42" customHeight="1" s="72"/>
+    <row r="19" ht="42" customHeight="1" s="72"/>
+    <row r="20" ht="42" customHeight="1" s="72"/>
+    <row r="21" ht="42" customHeight="1" s="72"/>
+    <row r="22" ht="42" customHeight="1" s="72"/>
+    <row r="23" ht="15.75" customHeight="1" s="72"/>
+    <row r="24" ht="22" customHeight="1" s="72"/>
+    <row r="25" ht="15.75" customHeight="1" s="72"/>
+    <row r="26" ht="15.75" customHeight="1" s="72"/>
+    <row r="27" ht="15.75" customHeight="1" s="72"/>
+    <row r="28" ht="15.75" customHeight="1" s="72"/>
     <row r="29" ht="15.75" customHeight="1" s="72"/>
     <row r="30" ht="15.75" customHeight="1" s="72"/>
     <row r="31" ht="15.75" customHeight="1" s="72"/>

</xml_diff>

<commit_message>
tracker: limpiar watchlist 9-Jun — eliminar GOOG/FLXS, descartar Stage3/4, actualizar market direction 5 dist days
</commit_message>
<xml_diff>
--- a/CAN_SLIM_Tracker_updated.xlsx
+++ b/CAN_SLIM_Tracker_updated.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 Watchlist Activa" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔬 DeepSeek Fase 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Revisiones MCP Hoy" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📈 Historial Operaciones" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚙️ Estado Sistema" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="🎯 Watchlist Activa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="🔬 DeepSeek Fase 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📊 Revisiones MCP Hoy" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="📈 Historial Operaciones" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="⚙️ Estado Sistema" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +80,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +132,12 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -159,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -228,6 +234,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -595,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -628,7 +643,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Market Direction: ALCISTA ✅  |  Distribution Days: 4/5 ⚠️  |  FTD: No confirmado  |  Screener: 20 finalistas | DeepSeek Fase 2: 6 analizados | APROBADOS Fase 3: 0</t>
+          <t>Market Direction: DISTRIBUCIÓN ⚠️  |  Distribution Days: 5/5 🔴  |  FTD: No confirmado  |  Actualizado: 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -1108,150 +1123,150 @@
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>PARR</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Par Pacific Holdings, Inc.</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="24" t="n">
         <v>57.1</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="24" t="n">
         <v>99</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="24" t="n">
         <v>279.1</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="24" t="n">
         <v>4.5</v>
       </c>
-      <c r="I10" s="10" t="inlineStr">
+      <c r="I10" s="24" t="inlineStr">
         <is>
           <t>INVALIDO</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>STAGE_3_DISTRIBUTION_RISK</t>
         </is>
       </c>
-      <c r="K10" s="10" t="inlineStr">
+      <c r="K10" s="24" t="inlineStr">
         <is>
           <t>NO_CLEAR_BASE</t>
         </is>
       </c>
-      <c r="L10" s="10" t="n">
+      <c r="L10" s="24" t="n">
         <v>70.39</v>
       </c>
-      <c r="M10" s="10" t="n">
+      <c r="M10" s="24" t="n">
         <v>-18.9</v>
       </c>
-      <c r="N10" s="10" t="n">
+      <c r="N10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="O10" s="10" t="n">
+      <c r="O10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="P10" s="10" t="inlineStr">
+      <c r="P10" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q10" s="10" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R10" s="12" t="inlineStr">
-        <is>
-          <t>Sin análisis adicional hoy.</t>
+      <c r="Q10" s="24" t="inlineStr">
+        <is>
+          <t>🚫 DESCARTAR</t>
+        </is>
+      </c>
+      <c r="R10" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>VAL</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Valaris Limited</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="24" t="n">
         <v>93.48</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="24" t="n">
         <v>99</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="24" t="n">
         <v>56.7</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="24" t="n">
         <v>-25</v>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="24" t="inlineStr">
         <is>
           <t>INVALIDO</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>STAGE_3_DISTRIBUTION_RISK</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="K11" s="24" t="inlineStr">
         <is>
           <t>NO_CLEAR_BASE</t>
         </is>
       </c>
-      <c r="L11" s="7" t="n">
+      <c r="L11" s="24" t="n">
         <v>114.12</v>
       </c>
-      <c r="M11" s="7" t="n">
+      <c r="M11" s="24" t="n">
         <v>-18.1</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="N11" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="O11" s="7" t="n">
+      <c r="O11" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="P11" s="7" t="inlineStr">
+      <c r="P11" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q11" s="7" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R11" s="9" t="inlineStr">
-        <is>
-          <t>Sin análisis adicional hoy.</t>
+      <c r="Q11" s="24" t="inlineStr">
+        <is>
+          <t>🚫 DESCARTAR</t>
+        </is>
+      </c>
+      <c r="R11" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
         </is>
       </c>
     </row>
@@ -1478,76 +1493,76 @@
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>BVN</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>Compañía de Minas Buenaventura S.A.A.</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>Basic Materials</t>
         </is>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="24" t="n">
         <v>35.15</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="24" t="n">
         <v>98</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="24" t="n">
         <v>1041.2</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="24" t="n">
         <v>108.1</v>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="24" t="inlineStr">
         <is>
           <t>INVALIDO</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>STAGE_1_OR_TRANSITION</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K15" s="24" t="inlineStr">
         <is>
           <t>CUP_OR_RECOVERY_BASE</t>
         </is>
       </c>
-      <c r="L15" s="7" t="n">
+      <c r="L15" s="24" t="n">
         <v>43.41</v>
       </c>
-      <c r="M15" s="7" t="n">
+      <c r="M15" s="24" t="n">
         <v>-19</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="O15" s="7" t="n">
+      <c r="O15" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="P15" s="7" t="inlineStr">
+      <c r="P15" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q15" s="7" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R15" s="9" t="inlineStr">
-        <is>
-          <t>Spike rechazado. Etapa 1/transición. Esperar base 6-8 semanas.</t>
+      <c r="Q15" s="24" t="inlineStr">
+        <is>
+          <t>🚫 DESCARTAR</t>
+        </is>
+      </c>
+      <c r="R15" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
         </is>
       </c>
     </row>
@@ -1626,148 +1641,148 @@
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Alphabet Inc.</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>372.58</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>95</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>81.2</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>ESPERAR</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>DAN</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Dana Incorporated</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F17" s="24" t="n">
+        <v>91</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>4248</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>INVALIDO</t>
+        </is>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>STAGE_3_DISTRIBUTION_RISK</t>
+        </is>
+      </c>
+      <c r="K17" s="24" t="inlineStr">
+        <is>
+          <t>CUP_OR_RECOVERY_BASE</t>
+        </is>
+      </c>
+      <c r="L17" s="24" t="n">
+        <v>39.42</v>
+      </c>
+      <c r="M17" s="24" t="n">
+        <v>-12.2</v>
+      </c>
+      <c r="N17" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="P17" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q17" s="24" t="inlineStr">
+        <is>
+          <t>🚫 DESCARTAR</t>
+        </is>
+      </c>
+      <c r="R17" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>LPG</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Dorian LPG Ltd.</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>41.31</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>91</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>901.2</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>102</v>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>INVALIDO</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>STAGE_2_ADVANCE</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
-        <is>
-          <t>HANDLE_OR_VCP_TIGHTENING</t>
-        </is>
-      </c>
-      <c r="L17" s="7" t="n">
-        <v>404.47</v>
-      </c>
-      <c r="M17" s="7" t="n">
-        <v>-7.9</v>
-      </c>
-      <c r="N17" s="7" t="n">
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>NO_CLEAR_BASE</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>48.12</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>-14.2</v>
+      </c>
+      <c r="N18" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="O17" s="7" t="n">
+      <c r="O18" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="P17" s="7" t="inlineStr">
-        <is>
-          <t>REVISAR (65)</t>
-        </is>
-      </c>
-      <c r="Q17" s="7" t="inlineStr">
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q18" s="7" t="inlineStr">
         <is>
           <t>👀 WATCHLIST</t>
         </is>
       </c>
-      <c r="R17" s="9" t="inlineStr">
-        <is>
-          <t>DeepSeek REVISAR 65. Pivot -7.9%. RS no confirmada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>DAN</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Dana Incorporated</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>34.6</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>91</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>4248</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>INVALIDO</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>STAGE_3_DISTRIBUTION_RISK</t>
-        </is>
-      </c>
-      <c r="K18" s="10" t="inlineStr">
-        <is>
-          <t>CUP_OR_RECOVERY_BASE</t>
-        </is>
-      </c>
-      <c r="L18" s="10" t="n">
-        <v>39.42</v>
-      </c>
-      <c r="M18" s="10" t="n">
-        <v>-12.2</v>
-      </c>
-      <c r="N18" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="O18" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="P18" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q18" s="10" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R18" s="12" t="inlineStr">
+      <c r="R18" s="9" t="inlineStr">
         <is>
           <t>Sin análisis adicional hoy.</t>
         </is>
@@ -1779,34 +1794,34 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>LPG</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Dorian LPG Ltd.</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>41.31</v>
+        <v>224.36</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>901.2</v>
+        <v>210.6</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>102</v>
+        <v>85.2</v>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>INVALIDO</t>
+          <t>ESPERAR</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
@@ -1816,14 +1831,14 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>NO_CLEAR_BASE</t>
+          <t>HANDLE_OR_VCP_TIGHTENING</t>
         </is>
       </c>
       <c r="L19" s="7" t="n">
-        <v>48.12</v>
+        <v>236.54</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>-14.2</v>
+        <v>-5.1</v>
       </c>
       <c r="N19" s="7" t="n">
         <v>3</v>
@@ -1833,390 +1848,244 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
+          <t>REVISAR (65)</t>
+        </is>
+      </c>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>👀 WATCHLIST</t>
+        </is>
+      </c>
+      <c r="R19" s="9" t="inlineStr">
+        <is>
+          <t>DeepSeek REVISAR 65. Pivot -5.1%. RS no confirmada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>OR Royalties Inc.</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="n">
+        <v>35.95</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <v>52</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <v>187</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <v>87.3</v>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>INVALIDO</t>
+        </is>
+      </c>
+      <c r="J20" s="24" t="inlineStr">
+        <is>
+          <t>STAGE_3_DISTRIBUTION_RISK</t>
+        </is>
+      </c>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>NO_CLEAR_BASE</t>
+        </is>
+      </c>
+      <c r="L20" s="24" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="M20" s="24" t="n">
+        <v>-25.1</v>
+      </c>
+      <c r="N20" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" s="24" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q19" s="7" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R19" s="9" t="inlineStr">
-        <is>
-          <t>Sin análisis adicional hoy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>FLXS</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Flexsteel Industries, Inc.</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>58.06</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>86</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>272.2</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>ESPERAR</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
+      <c r="Q20" s="24" t="inlineStr">
+        <is>
+          <t>🚫 DESCARTAR</t>
+        </is>
+      </c>
+      <c r="R20" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>SLDE</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Slide Insurance Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="n">
+        <v>17.83</v>
+      </c>
+      <c r="F21" s="24" t="n">
+        <v>29</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="H21" s="24" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>INVALIDO</t>
+        </is>
+      </c>
+      <c r="J21" s="24" t="inlineStr">
+        <is>
+          <t>STAGE_3_DISTRIBUTION_RISK</t>
+        </is>
+      </c>
+      <c r="K21" s="24" t="inlineStr">
+        <is>
+          <t>HANDLE_OR_VCP_TIGHTENING</t>
+        </is>
+      </c>
+      <c r="L21" s="24" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="M21" s="24" t="n">
+        <v>-31.2</v>
+      </c>
+      <c r="N21" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O21" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="P21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q21" s="24" t="inlineStr">
+        <is>
+          <t>🚫 DESCARTAR</t>
+        </is>
+      </c>
+      <c r="R21" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="25" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>Vistance Networks, Inc.</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="F22" s="24" t="n">
+        <v>99</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>602.6</v>
+      </c>
+      <c r="H22" s="24" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="I22" s="24" t="inlineStr">
+        <is>
+          <t>INVALIDO</t>
+        </is>
+      </c>
+      <c r="J22" s="24" t="inlineStr">
         <is>
           <t>STAGE_2_ADVANCE</t>
         </is>
       </c>
-      <c r="K20" s="10" t="inlineStr">
-        <is>
-          <t>CUP_OR_RECOVERY_BASE</t>
-        </is>
-      </c>
-      <c r="L20" s="10" t="n">
-        <v>60.97</v>
-      </c>
-      <c r="M20" s="10" t="n">
-        <v>-4.8</v>
-      </c>
-      <c r="N20" s="10" t="n">
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>NO_CLEAR_BASE</t>
+        </is>
+      </c>
+      <c r="L22" s="24" t="n">
+        <v>13.22</v>
+      </c>
+      <c r="M22" s="24" t="n">
+        <v>-7.2</v>
+      </c>
+      <c r="N22" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="O20" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="10" t="inlineStr">
-        <is>
-          <t>REVISAR (65)</t>
-        </is>
-      </c>
-      <c r="Q20" s="10" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R20" s="12" t="inlineStr">
-        <is>
-          <t>Sin análisis adicional hoy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>224.36</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>67</v>
-      </c>
-      <c r="G21" s="7" t="n">
-        <v>210.6</v>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>ESPERAR</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>STAGE_2_ADVANCE</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>HANDLE_OR_VCP_TIGHTENING</t>
-        </is>
-      </c>
-      <c r="L21" s="7" t="n">
-        <v>236.54</v>
-      </c>
-      <c r="M21" s="7" t="n">
-        <v>-5.1</v>
-      </c>
-      <c r="N21" s="7" t="n">
+      <c r="O22" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="O21" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="P21" s="7" t="inlineStr">
-        <is>
-          <t>REVISAR (65)</t>
-        </is>
-      </c>
-      <c r="Q21" s="7" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R21" s="9" t="inlineStr">
-        <is>
-          <t>DeepSeek REVISAR 65. Pivot -5.1%. RS no confirmada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>OR Royalties Inc.</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>Basic Materials</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="n">
-        <v>35.95</v>
-      </c>
-      <c r="F22" s="10" t="n">
-        <v>52</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>187</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>87.3</v>
-      </c>
-      <c r="I22" s="10" t="inlineStr">
-        <is>
-          <t>INVALIDO</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
-        <is>
-          <t>STAGE_3_DISTRIBUTION_RISK</t>
-        </is>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>NO_CLEAR_BASE</t>
-        </is>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="M22" s="10" t="n">
-        <v>-25.1</v>
-      </c>
-      <c r="N22" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="O22" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="P22" s="10" t="inlineStr">
+      <c r="P22" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q22" s="10" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R22" s="12" t="inlineStr">
-        <is>
-          <t>Sin análisis adicional hoy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>SLDE</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Slide Insurance Holdings, Inc.</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Financial Services</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>17.83</v>
-      </c>
-      <c r="F23" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="G23" s="7" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="H23" s="7" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>INVALIDO</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>STAGE_3_DISTRIBUTION_RISK</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>HANDLE_OR_VCP_TIGHTENING</t>
-        </is>
-      </c>
-      <c r="L23" s="7" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="M23" s="7" t="n">
-        <v>-31.2</v>
-      </c>
-      <c r="N23" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="O23" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="P23" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q23" s="7" t="inlineStr">
-        <is>
-          <t>👀 WATCHLIST</t>
-        </is>
-      </c>
-      <c r="R23" s="9" t="inlineStr">
-        <is>
-          <t>Sin análisis adicional hoy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>VISN</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Vistance Networks, Inc.</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="n">
-        <v>12.27</v>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>99</v>
-      </c>
-      <c r="G24" s="13" t="n">
-        <v>602.6</v>
-      </c>
-      <c r="H24" s="13" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="I24" s="13" t="inlineStr">
-        <is>
-          <t>INVALIDO</t>
-        </is>
-      </c>
-      <c r="J24" s="13" t="inlineStr">
-        <is>
-          <t>STAGE_2_ADVANCE</t>
-        </is>
-      </c>
-      <c r="K24" s="13" t="inlineStr">
-        <is>
-          <t>NO_CLEAR_BASE</t>
-        </is>
-      </c>
-      <c r="L24" s="13" t="n">
-        <v>13.22</v>
-      </c>
-      <c r="M24" s="13" t="n">
-        <v>-7.2</v>
-      </c>
-      <c r="N24" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="O24" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="P24" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q22" s="24" t="inlineStr">
         <is>
           <t>🚫 DESCARTAR</t>
         </is>
       </c>
-      <c r="R24" s="15" t="inlineStr">
-        <is>
-          <t>Death cross confirmado MCP. Volumen 50K. Sacar de watchlist.</t>
-        </is>
-      </c>
-    </row>
+      <c r="R22" s="26" t="inlineStr">
+        <is>
+          <t>Stage 3/4 — distribución confirmada. Eliminado de watchlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1"/>
+    <row r="24" ht="40" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:R2"/>

</xml_diff>